<commit_message>
contemplar libres de contenedores
</commit_message>
<xml_diff>
--- a/tests/manifiesto_prueba.xlsx
+++ b/tests/manifiesto_prueba.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -866,6 +866,132 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DHEAM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UYMVD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>S329701796</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>40HC</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>40HC</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Consolidated Shipments stc 55 pkgs spare parts</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>GCNU4865094</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Jauser Soluciones Logisticas</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>1714</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>5</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DHEAM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UYMVD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>S329701796</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>40HC</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>40HC</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Consolidated Shipments stc 44 pkgs spare parts</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ACLU9803492</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Jauser Soluciones Logisticas</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>1714</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrupar filas 1716 del mismo BL en un solo PDF.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/manifiesto_prueba.xlsx
+++ b/tests/manifiesto_prueba.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -810,122 +810,122 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BRPNS</t>
+          <t>DHEAM</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BRPNS</t>
+          <t>UYMVD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>S329509809</t>
+          <t>S329568298</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>USED LM ROROUroro</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>VEH</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>VEH</t>
-        </is>
-      </c>
       <c r="F8" t="n">
-        <v>503</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>RENAULT</t>
+          <t>PORSCHE MACAN GTSPORSCHE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>WP1ZZZXAZTL251415</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>SANTA ROSA AUTOMOTORS</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>DD1651</t>
-        </is>
+          <t>Nordenwagen Uruguay Sa</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>1716</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DHEAM</t>
+          <t>BRPNS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UYMVD</t>
+          <t>BRPNS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>S329701796</t>
+          <t>S329509809</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>40HC</t>
+          <t>VEH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>40HC</t>
+          <t>VEH</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>503</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Consolidated Shipments stc 55 pkgs spare parts</t>
+          <t>RENAULT</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>GCNU4865094</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Jauser Soluciones Logisticas</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>1714</v>
+          <t>SANTA ROSA AUTOMOTORS</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>DD1651</t>
+        </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>5</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>28/08/2026</t>
-        </is>
-      </c>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
     </row>
@@ -960,12 +960,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Consolidated Shipments stc 44 pkgs spare parts</t>
+          <t>Consolidated Shipments stc 55 pkgs spare parts</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ACLU9803492</t>
+          <t>GCNU4865094</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -991,6 +991,69 @@
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DHEAM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UYMVD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>S329701796</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>40HC</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>40HC</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Consolidated Shipments stc 44 pkgs spare parts</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ACLU9803492</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Jauser Soluciones Logisticas</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>1714</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>